<commit_message>
Update game history: remove Genshin Impact and add osu!
</commit_message>
<xml_diff>
--- a/我的游戏游玩经历.xlsx
+++ b/我的游戏游玩经历.xlsx
@@ -675,39 +675,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>星露谷物语 Stardew Valley</t>
+          <t xml:space="preserve">osu!</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>模拟经营</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
+          <t xml:space="preserve">音乐节奏（音游）</t>
+        </is>
+      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>高中</t>
+          <t xml:space="preserve">初三暑假</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>持续游玩至今</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>长线农场经营</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>初中起就常看相关实况，高中正式入坑</t>
-        </is>
-      </c>
+          <t xml:space="preserve">三年</t>
+        </is>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -715,17 +703,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>宝可梦系列</t>
+          <t xml:space="preserve">星露谷物语 Stardew Valley</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>角色扮演/回合制</t>
+          <t xml:space="preserve">模拟经营</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>掌机/主机</t>
+          <t xml:space="preserve">PC</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -740,12 +728,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>系列多作持续跟进</t>
+          <t xml:space="preserve">长线农场经营</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t xml:space="preserve">初中起就常看相关实况，高中正式入坑</t>
         </is>
       </c>
     </row>
@@ -755,17 +743,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>崩坏：星穹铁道</t>
+          <t xml:space="preserve">宝可梦系列</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>回合制二次元</t>
+          <t xml:space="preserve">角色扮演/回合制</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>手机/PC</t>
+          <t xml:space="preserve">掌机/主机</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -780,7 +768,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>长期在线运营游戏，稳定跟版本</t>
+          <t xml:space="preserve">系列多作持续跟进</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -795,12 +783,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>原神</t>
+          <t xml:space="preserve">崩坏：星穹铁道</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>开放世界二次元</t>
+          <t xml:space="preserve">回合制二次元</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -820,7 +808,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>开放世界探索 + 版本跟进</t>
+          <t xml:space="preserve">长期在线运营游戏，稳定跟版本</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1099,12 +1087,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>饥荒、英雄无敌、泰拉瑞亚</t>
+          <t xml:space="preserve">饥荒、英雄无敌、泰拉瑞亚、osu!</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>偏单机：生存、策略、沙盒；同时开始看游戏实况</t>
+          <t xml:space="preserve">偏单机：生存、策略、沙盒；开始看游戏实况；初三暑假入坑 osu!，游玩三年</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1109,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>星露谷物语、宝可梦系列、崩坏：星穹铁道、原神</t>
+          <t xml:space="preserve">星露谷物语、宝可梦系列、崩坏：星穹铁道</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1209,7 +1197,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>星露谷、宝可梦、星穹铁道、原神 + 看实况</t>
+          <t xml:space="preserve">星露谷、宝可梦、星穹铁道 + 看实况</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1292,7 +1280,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>星露谷物语、宝可梦系列、崩坏：星穹铁道、原神</t>
+          <t xml:space="preserve">星露谷物语、宝可梦系列、崩坏：星穹铁道</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1304,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>沙盒建造、生存、回合制策略、模拟经营、角色扮演、二次元抽卡、FPS、MOBA、生存恐怖、剧情推理</t>
+          <t xml:space="preserve">沙盒建造、生存、回合制策略、模拟经营、角色扮演、二次元抽卡、FPS、MOBA、生存恐怖、剧情推理、音乐节奏</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Resident Evil and Witch Trial platforms to PC
</commit_message>
<xml_diff>
--- a/我的游戏游玩经历.xlsx
+++ b/我的游戏游玩经历.xlsx
@@ -913,7 +913,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>主机</t>
+          <t xml:space="preserve">PC</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>主机平台代表作之一</t>
+          <t xml:space="preserve">生存恐怖系列代表作之一</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -949,7 +949,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>主机</t>
+          <t xml:space="preserve">PC</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>转向主机游戏，偏剧情与单机体验</t>
+          <t xml:space="preserve">在 PC 上游玩，偏剧情与单机体验</t>
         </is>
       </c>
     </row>

</xml_diff>